<commit_message>
limpieza del script, error en trees Id corregido, revisando SLA pero se ven coherentes
</commit_message>
<xml_diff>
--- a/NUMEX_pre_RStudio/modelos_est.xlsx
+++ b/NUMEX_pre_RStudio/modelos_est.xlsx
@@ -65,13 +65,13 @@
     <t xml:space="preserve">(Intercept)</t>
   </si>
   <si>
-    <t xml:space="preserve">SUBN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUBNP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUBP</t>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N × P</t>
   </si>
   <si>
     <t xml:space="preserve">SD (Intercept Bloque)</t>
@@ -119,18 +119,18 @@
     <t xml:space="preserve">(0.579)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.780</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.592)</t>
-  </si>
-  <si>
     <t xml:space="preserve">1.320*</t>
   </si>
   <si>
     <t xml:space="preserve">(0.561)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.871</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.846)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.562</t>
   </si>
   <si>
@@ -164,18 +164,18 @@
     <t xml:space="preserve">(2.674)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.688*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.891)</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.227</t>
   </si>
   <si>
     <t xml:space="preserve">(1.769)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.794</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(3.206)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.000</t>
   </si>
   <si>
@@ -206,18 +206,18 @@
     <t xml:space="preserve">(0.689)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.429</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.713)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.508</t>
   </si>
   <si>
     <t xml:space="preserve">(0.605)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.482</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.971)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.562</t>
   </si>
   <si>
@@ -245,18 +245,18 @@
     <t xml:space="preserve">(0.415)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.777+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.386)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.979*</t>
   </si>
   <si>
     <t xml:space="preserve">(0.404)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.775</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.588)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.017</t>
   </si>
   <si>
@@ -284,18 +284,18 @@
     <t xml:space="preserve">(1.180)</t>
   </si>
   <si>
-    <t xml:space="preserve">2.589+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.421)</t>
-  </si>
-  <si>
     <t xml:space="preserve">1.359</t>
   </si>
   <si>
     <t xml:space="preserve">(1.131)</t>
   </si>
   <si>
+    <t xml:space="preserve">-2.174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1.778)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.417</t>
   </si>
   <si>
@@ -329,18 +329,18 @@
     <t xml:space="preserve">(0.989)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.739</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.308)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.297</t>
   </si>
   <si>
     <t xml:space="preserve">(0.947)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.590</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1.615)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.563</t>
   </si>
   <si>
@@ -368,15 +368,18 @@
     <t xml:space="preserve">(0.036)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.049</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.082*</t>
   </si>
   <si>
     <t xml:space="preserve">(0.034)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.052)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.038</t>
   </si>
   <si>
@@ -407,18 +410,18 @@
     <t xml:space="preserve">(0.146)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.289*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.103)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.120</t>
   </si>
   <si>
     <t xml:space="preserve">(0.097)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.175)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.127</t>
   </si>
   <si>
@@ -443,82 +446,82 @@
     <t xml:space="preserve">(0.060)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.084)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.135</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.159</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-25.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logNmass | 2000 | Myrcia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.188***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.029)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.110*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.045)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-0.110*</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.044)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.089</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.064)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.111</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.361</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-47.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">logNmass | 3000 | Hedyosmum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.648***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.065)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.201**</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.088</t>
+  </si>
+  <si>
     <t xml:space="preserve">(0.062)</t>
   </si>
   <si>
-    <t xml:space="preserve">-0.043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.052)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.135</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-25.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">logNmass | 2000 | Myrcia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.188***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.029)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.110*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.045)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.090*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.042)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-0.110*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.044)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.111</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.361</t>
-  </si>
-  <si>
-    <t xml:space="preserve">-47.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">logNmass | 3000 | Hedyosmum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.648***</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.065)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.201**</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.163+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.078)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.088</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.089</t>
+    <t xml:space="preserve">-0.126</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.098)</t>
   </si>
   <si>
     <t xml:space="preserve">0.106</t>
@@ -539,27 +542,24 @@
     <t xml:space="preserve">2.338***</t>
   </si>
   <si>
-    <t xml:space="preserve">(0.064)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.092</t>
   </si>
   <si>
     <t xml:space="preserve">(0.091)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.076</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.121)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.026</t>
   </si>
   <si>
     <t xml:space="preserve">(0.087)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.149)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.144</t>
   </si>
   <si>
@@ -578,18 +578,18 @@
     <t xml:space="preserve">(0.108)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.154</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.120)</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.250*</t>
   </si>
   <si>
     <t xml:space="preserve">(0.115)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.222</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.168)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.248</t>
   </si>
   <si>
@@ -614,15 +614,15 @@
     <t xml:space="preserve">(0.236)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.322</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.167)</t>
-  </si>
-  <si>
     <t xml:space="preserve">(0.156)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.266</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.283)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.204</t>
   </si>
   <si>
@@ -647,18 +647,18 @@
     <t xml:space="preserve">(0.264)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.031</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.274)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.158</t>
   </si>
   <si>
     <t xml:space="preserve">(0.232)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.248</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.373)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.600</t>
   </si>
   <si>
@@ -683,15 +683,15 @@
     <t xml:space="preserve">(0.151)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.330*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.140)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.120</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.213)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.369</t>
   </si>
   <si>
@@ -716,18 +716,18 @@
     <t xml:space="preserve">(0.222)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.448</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.268)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.022</t>
   </si>
   <si>
     <t xml:space="preserve">(0.214)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.232</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(0.336)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.094</t>
   </si>
   <si>
@@ -758,18 +758,15 @@
     <t xml:space="preserve">(0.144)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.069</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(0.191)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.000</t>
   </si>
   <si>
     <t xml:space="preserve">(0.138)</t>
   </si>
   <si>
+    <t xml:space="preserve">-0.113</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.228</t>
   </si>
   <si>
@@ -794,18 +791,18 @@
     <t xml:space="preserve">(7.962)</t>
   </si>
   <si>
-    <t xml:space="preserve">-2.147</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(8.663)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-0.616</t>
   </si>
   <si>
     <t xml:space="preserve">(8.293)</t>
   </si>
   <si>
+    <t xml:space="preserve">1.207</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(12.169)</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.663</t>
   </si>
   <si>
@@ -833,13 +830,16 @@
     <t xml:space="preserve">(15.767)</t>
   </si>
   <si>
-    <t xml:space="preserve">9.125</t>
+    <t xml:space="preserve">16.973</t>
   </si>
   <si>
     <t xml:space="preserve">(10.429)</t>
   </si>
   <si>
-    <t xml:space="preserve">16.973</t>
+    <t xml:space="preserve">-33.621</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(18.489)</t>
   </si>
   <si>
     <t xml:space="preserve">13.655</t>
@@ -869,18 +869,18 @@
     <t xml:space="preserve">(6.247)</t>
   </si>
   <si>
-    <t xml:space="preserve">-8.613</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(6.466)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-4.799</t>
   </si>
   <si>
     <t xml:space="preserve">(5.486)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(8.802)</t>
+  </si>
+  <si>
     <t xml:space="preserve">14.166</t>
   </si>
   <si>
@@ -905,18 +905,18 @@
     <t xml:space="preserve">(3.198)</t>
   </si>
   <si>
-    <t xml:space="preserve">-7.745*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(3.032)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-4.308</t>
   </si>
   <si>
     <t xml:space="preserve">(3.128)</t>
   </si>
   <si>
+    <t xml:space="preserve">-1.931</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(4.575)</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.695</t>
   </si>
   <si>
@@ -944,18 +944,18 @@
     <t xml:space="preserve">(4.459)</t>
   </si>
   <si>
-    <t xml:space="preserve">4.616</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(5.373)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-1.430</t>
   </si>
   <si>
     <t xml:space="preserve">(4.301)</t>
   </si>
   <si>
+    <t xml:space="preserve">9.399</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(6.746)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.848</t>
   </si>
   <si>
@@ -986,18 +986,18 @@
     <t xml:space="preserve">(6.780)</t>
   </si>
   <si>
-    <t xml:space="preserve">17.429+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(9.040)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-2.611</t>
   </si>
   <si>
     <t xml:space="preserve">(6.503)</t>
   </si>
   <si>
+    <t xml:space="preserve">19.142</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11.017)</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.022</t>
   </si>
   <si>
@@ -1028,18 +1028,18 @@
     <t xml:space="preserve">(4.007)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.288</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4.434)</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.011</t>
   </si>
   <si>
     <t xml:space="preserve">(4.261)</t>
   </si>
   <si>
+    <t xml:space="preserve">-4.105</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(6.211)</t>
+  </si>
+  <si>
     <t xml:space="preserve">9.170</t>
   </si>
   <si>
@@ -1064,18 +1064,18 @@
     <t xml:space="preserve">(2.642)</t>
   </si>
   <si>
-    <t xml:space="preserve">-5.063*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.656)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-2.305</t>
   </si>
   <si>
     <t xml:space="preserve">(1.759)</t>
   </si>
   <si>
+    <t xml:space="preserve">5.705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(3.381)</t>
+  </si>
+  <si>
     <t xml:space="preserve">3.690</t>
   </si>
   <si>
@@ -1103,18 +1103,18 @@
     <t xml:space="preserve">(6.980)</t>
   </si>
   <si>
-    <t xml:space="preserve">-6.643</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(7.172)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-3.840</t>
   </si>
   <si>
     <t xml:space="preserve">(6.087)</t>
   </si>
   <si>
+    <t xml:space="preserve">-2.296</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(9.813)</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.062</t>
   </si>
   <si>
@@ -1145,18 +1145,18 @@
     <t xml:space="preserve">(5.778)</t>
   </si>
   <si>
-    <t xml:space="preserve">3.656</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(5.395)</t>
-  </si>
-  <si>
     <t xml:space="preserve">8.640</t>
   </si>
   <si>
     <t xml:space="preserve">(5.628)</t>
   </si>
   <si>
+    <t xml:space="preserve">-13.686</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(8.209)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.939</t>
   </si>
   <si>
@@ -1187,18 +1187,18 @@
     <t xml:space="preserve">(6.687)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.796</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(8.065)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-7.692</t>
   </si>
   <si>
     <t xml:space="preserve">(6.467)</t>
   </si>
   <si>
+    <t xml:space="preserve">2.922</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(10.139)</t>
+  </si>
+  <si>
     <t xml:space="preserve">11.044</t>
   </si>
   <si>
@@ -1223,16 +1223,16 @@
     <t xml:space="preserve">(3.981)</t>
   </si>
   <si>
-    <t xml:space="preserve">0.233</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(5.266)</t>
-  </si>
-  <si>
     <t xml:space="preserve">-2.826</t>
   </si>
   <si>
     <t xml:space="preserve">(3.812)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.675</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(6.501)</t>
   </si>
   <si>
     <t xml:space="preserve">6.295</t>
@@ -2037,230 +2037,230 @@
         <v>118</v>
       </c>
       <c r="G10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H10" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I10" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J10" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="K10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="L10" t="s">
         <v>41</v>
       </c>
       <c r="M10" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="N10" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="O10" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D11" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F11" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G11" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I11" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J11" t="s">
         <v>54</v>
       </c>
       <c r="K11" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="L11" t="s">
         <v>56</v>
       </c>
       <c r="M11" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="N11" t="s">
         <v>29</v>
       </c>
       <c r="O11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E12" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F12" t="s">
+        <v>144</v>
+      </c>
+      <c r="G12" t="s">
         <v>121</v>
       </c>
-      <c r="G12" t="s">
-        <v>143</v>
-      </c>
       <c r="H12" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J12" t="s">
         <v>54</v>
       </c>
       <c r="K12" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="L12" t="s">
         <v>69</v>
       </c>
       <c r="M12" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="N12" t="s">
         <v>29</v>
       </c>
       <c r="O12" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D13" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H13" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J13" t="s">
         <v>54</v>
       </c>
       <c r="K13" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L13" t="s">
         <v>82</v>
       </c>
       <c r="M13" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="N13" t="s">
         <v>29</v>
       </c>
       <c r="O13" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B14" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C14" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D14" t="s">
+        <v>165</v>
+      </c>
+      <c r="E14" t="s">
         <v>164</v>
       </c>
-      <c r="E14" t="s">
-        <v>163</v>
-      </c>
       <c r="F14" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G14" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H14" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I14" t="s">
-        <v>143</v>
+        <v>169</v>
       </c>
       <c r="J14" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="K14" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L14" t="s">
         <v>96</v>
       </c>
       <c r="M14" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N14" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="O14" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B15" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C15" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="D15" t="s">
         <v>176</v>
@@ -2310,7 +2310,7 @@
         <v>186</v>
       </c>
       <c r="D16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E16" t="s">
         <v>187</v>
@@ -2363,13 +2363,13 @@
         <v>199</v>
       </c>
       <c r="F17" t="s">
+        <v>148</v>
+      </c>
+      <c r="G17" t="s">
         <v>200</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>201</v>
-      </c>
-      <c r="H17" t="s">
-        <v>147</v>
       </c>
       <c r="I17" t="s">
         <v>202</v>
@@ -2460,13 +2460,13 @@
         <v>223</v>
       </c>
       <c r="G19" t="s">
+        <v>131</v>
+      </c>
+      <c r="H19" t="s">
         <v>224</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>225</v>
-      </c>
-      <c r="I19" t="s">
-        <v>130</v>
       </c>
       <c r="J19" t="s">
         <v>54</v>
@@ -2560,101 +2560,101 @@
         <v>250</v>
       </c>
       <c r="I21" t="s">
-        <v>251</v>
+        <v>199</v>
       </c>
       <c r="J21" t="s">
         <v>54</v>
       </c>
       <c r="K21" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="L21" t="s">
         <v>110</v>
       </c>
       <c r="M21" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="N21" t="s">
         <v>29</v>
       </c>
       <c r="O21" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
+        <v>254</v>
+      </c>
+      <c r="B22" t="s">
         <v>255</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>256</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>257</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>258</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>259</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>260</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>261</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>262</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>263</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>264</v>
-      </c>
-      <c r="K22" t="s">
-        <v>265</v>
       </c>
       <c r="L22" t="s">
         <v>41</v>
       </c>
       <c r="M22" t="s">
+        <v>265</v>
+      </c>
+      <c r="N22" t="s">
+        <v>178</v>
+      </c>
+      <c r="O22" t="s">
         <v>266</v>
-      </c>
-      <c r="N22" t="s">
-        <v>180</v>
-      </c>
-      <c r="O22" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
+        <v>267</v>
+      </c>
+      <c r="B23" t="s">
         <v>268</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>269</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>270</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>271</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>272</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>273</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>274</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>275</v>
-      </c>
-      <c r="I23" t="s">
-        <v>274</v>
       </c>
       <c r="J23" t="s">
         <v>54</v>
@@ -2968,7 +2968,7 @@
         <v>361</v>
       </c>
       <c r="D30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E30" t="s">
         <v>362</v>

</xml_diff>